<commit_message>
Version 2.4.2.0 se agrego que al momento de cmabiar la guia usando codigo barras se guarde en una columna nueva la fecha de ese registro
</commit_message>
<xml_diff>
--- a/Jeic/Jeic/Resources/Plantilla.xlsx
+++ b/Jeic/Jeic/Resources/Plantilla.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\boxbu\source\repos\Axdrox\proyectoJeic\Jeic\Jeic\Resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\boxbu\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17596D62-2C53-43AA-85EC-91080C9368EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88931A8D-41CC-40FA-82F0-EB725507028F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plantilla" sheetId="1" r:id="rId1"/>
@@ -107,9 +107,6 @@
     <t>FECHA DEVOLUCIÓN</t>
   </si>
   <si>
-    <t>MOTIVO DE DEVOLUCIÓN</t>
-  </si>
-  <si>
     <t>CANTIDAD DE PIEZAS DEVUELTAS</t>
   </si>
   <si>
@@ -204,6 +201,9 @@
   </si>
   <si>
     <t>ESTADO DEL VALE</t>
+  </si>
+  <si>
+    <t>FECHA DE ENVÍO</t>
   </si>
 </sst>
 </file>
@@ -746,7 +746,7 @@
     </row>
     <row r="3" spans="1:54" x14ac:dyDescent="0.3">
       <c r="F3" s="15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G3" s="15"/>
       <c r="H3" s="15"/>
@@ -771,10 +771,10 @@
         <v>5</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H8" s="7" t="s">
         <v>6</v>
@@ -783,19 +783,19 @@
         <v>7</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="K8" s="7" t="s">
         <v>8</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="M8" s="7" t="s">
         <v>9</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="O8" s="7" t="s">
         <v>10</v>
@@ -807,7 +807,7 @@
         <v>12</v>
       </c>
       <c r="R8" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="S8" s="3" t="s">
         <v>13</v>
@@ -816,7 +816,7 @@
         <v>14</v>
       </c>
       <c r="U8" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="V8" s="10" t="s">
         <v>15</v>
@@ -846,81 +846,81 @@
         <v>23</v>
       </c>
       <c r="AE8" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="AF8" s="7" t="s">
+      <c r="AG8" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="AH8" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI8" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="AJ8" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AG8" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="AH8" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="AI8" s="7" t="s">
+      <c r="AK8" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="AL8" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="AM8" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="AN8" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="AO8" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="AP8" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="AQ8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="AR8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="AS8" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="AJ8" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="AK8" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="AL8" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="AM8" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="AN8" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="AO8" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="AP8" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="AQ8" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="AR8" s="7" t="s">
+      <c r="AT8" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="AS8" s="7" t="s">
+      <c r="AU8" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AV8" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AW8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="AX8" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="AY8" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="AZ8" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="AT8" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="AU8" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="AV8" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="AW8" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="AX8" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="AY8" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="AZ8" s="8" t="s">
+      <c r="BA8" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="BA8" s="7" t="s">
+      <c r="BB8" s="7" t="s">
         <v>55</v>
-      </c>
-      <c r="BB8" s="7" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:54" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Version 2.5.4.0 Se agrego el estado de REEMBOLSO y se cambio la columna (AA) del reporte por Realizo Baja
</commit_message>
<xml_diff>
--- a/Jeic/Jeic/Resources/Plantilla.xlsx
+++ b/Jeic/Jeic/Resources/Plantilla.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\boxbu\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88931A8D-41CC-40FA-82F0-EB725507028F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09CA0671-9155-46F3-8043-A1558621FC92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -95,9 +95,6 @@
     <t>PIEZAS ENTREGADAS</t>
   </si>
   <si>
-    <t>ENTREGA EN TIEMPO</t>
-  </si>
-  <si>
     <t>DÍAS DE ENTREGA</t>
   </si>
   <si>
@@ -204,6 +201,9 @@
   </si>
   <si>
     <t>FECHA DE ENVÍO</t>
+  </si>
+  <si>
+    <t>REALIZÓ BAJA</t>
   </si>
 </sst>
 </file>
@@ -746,7 +746,7 @@
     </row>
     <row r="3" spans="1:54" x14ac:dyDescent="0.3">
       <c r="F3" s="15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G3" s="15"/>
       <c r="H3" s="15"/>
@@ -771,10 +771,10 @@
         <v>5</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H8" s="7" t="s">
         <v>6</v>
@@ -783,19 +783,19 @@
         <v>7</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="K8" s="7" t="s">
         <v>8</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="M8" s="7" t="s">
         <v>9</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="O8" s="7" t="s">
         <v>10</v>
@@ -807,7 +807,7 @@
         <v>12</v>
       </c>
       <c r="R8" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="S8" s="3" t="s">
         <v>13</v>
@@ -816,7 +816,7 @@
         <v>14</v>
       </c>
       <c r="U8" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="V8" s="10" t="s">
         <v>15</v>
@@ -828,99 +828,99 @@
         <v>17</v>
       </c>
       <c r="Y8" s="14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Z8" s="7" t="s">
         <v>19</v>
       </c>
       <c r="AA8" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB8" s="7" t="s">
         <v>20</v>
-      </c>
-      <c r="AB8" s="7" t="s">
-        <v>21</v>
       </c>
       <c r="AC8" s="14" t="s">
         <v>18</v>
       </c>
       <c r="AD8" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="AE8" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="AF8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="AE8" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="AF8" s="7" t="s">
+      <c r="AG8" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="AH8" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="AI8" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="AJ8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="AG8" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="AH8" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="AI8" s="7" t="s">
+      <c r="AK8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="AL8" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="AM8" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="AN8" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="AO8" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="AP8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="AQ8" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="AR8" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="AS8" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="AJ8" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="AK8" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="AL8" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="AM8" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="AN8" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="AO8" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="AP8" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="AQ8" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="AR8" s="7" t="s">
+      <c r="AT8" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="AS8" s="7" t="s">
+      <c r="AU8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="AV8" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AW8" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="AX8" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="AY8" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="AZ8" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="AT8" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="AU8" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="AV8" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="AW8" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="AX8" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="AY8" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="AZ8" s="8" t="s">
+      <c r="BA8" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="BA8" s="7" t="s">
+      <c r="BB8" s="7" t="s">
         <v>54</v>
-      </c>
-      <c r="BB8" s="7" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:54" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se actualizo el Logo del Reporte de Ventas a JSO
</commit_message>
<xml_diff>
--- a/Jeic/Jeic/Resources/Plantilla.xlsx
+++ b/Jeic/Jeic/Resources/Plantilla.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\boxbu\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/de8a898b81206ef9/Documents/JSO REFACCIONARIA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09CA0671-9155-46F3-8043-A1558621FC92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{09CA0671-9155-46F3-8043-A1558621FC92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8381A92-5AE1-457C-AA48-45CBCAA2D124}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plantilla" sheetId="1" r:id="rId1"/>
@@ -373,15 +373,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:colOff>401001</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>733425</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>179069</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -395,15 +395,20 @@
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="114300" y="123825"/>
-          <a:ext cx="2514600" cy="781050"/>
+          <a:off x="401001" y="0"/>
+          <a:ext cx="2104074" cy="1264919"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>